<commit_message>
Improve filtering and import usability
</commit_message>
<xml_diff>
--- a/public/templates/OpsTracker_Import_Template.xlsx
+++ b/public/templates/OpsTracker_Import_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eugenehorfilla/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eugenehorfilla/github/opstracker/public/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B008CA8E-9B78-AB48-A1C5-A20D45BD4997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43E172C3-6DF4-6C47-AC51-5305DF7131E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="26600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="26600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Technical Assistance" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="35">
   <si>
     <t>Date</t>
   </si>
@@ -66,9 +66,6 @@
   </si>
   <si>
     <t>Remarks</t>
-  </si>
-  <si>
-    <t>2026-09-16</t>
   </si>
   <si>
     <t>MCR</t>
@@ -135,6 +132,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -181,10 +181,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -555,44 +556,44 @@
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="3">
+        <v>46289</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>16</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>18</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>19</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>20</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>21</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>22</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>23</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>24</v>
       </c>
-      <c r="L2" t="s">
+      <c r="O2" t="s">
         <v>25</v>
-      </c>
-      <c r="O2" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -634,10 +635,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>8</v>
@@ -662,38 +663,38 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="3">
+        <v>46289</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>16</v>
       </c>
-      <c r="D2" t="s">
-        <v>17</v>
-      </c>
       <c r="E2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" t="s">
         <v>29</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>30</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>31</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J2" t="s">
         <v>32</v>
       </c>
-      <c r="I2" t="s">
-        <v>24</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="M2" t="s">
         <v>33</v>
-      </c>
-      <c r="M2" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(import-export): support workbook-wide import, assignee mapping, and worklog exports
</commit_message>
<xml_diff>
--- a/public/templates/OpsTracker_Import_Template.xlsx
+++ b/public/templates/OpsTracker_Import_Template.xlsx
@@ -1,27 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eugenehorfilla/github/opstracker/public/templates/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43E172C3-6DF4-6C47-AC51-5305DF7131E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="26600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="26600"/>
   </bookViews>
   <sheets>
-    <sheet name="Technical Assistance" sheetId="1" r:id="rId1"/>
-    <sheet name="Other Tasks" sheetId="2" r:id="rId2"/>
+    <sheet sheetId="1" name="Technical Assistance" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Other Tasks" state="visible" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="36">
   <si>
     <t>Date</t>
   </si>
@@ -68,6 +62,12 @@
     <t>Remarks</t>
   </si>
   <si>
+    <t>End Date</t>
+  </si>
+  <si>
+    <t>10PM -6AM</t>
+  </si>
+  <si>
     <t>MCR</t>
   </si>
   <si>
@@ -123,32 +123,29 @@
   </si>
   <si>
     <t>Completed</t>
-  </si>
-  <si>
-    <t>10PM -6AM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
+      <family val="2"/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -184,14 +181,14 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -487,9 +484,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
@@ -506,9 +503,10 @@
     <col min="13" max="13" width="19" customWidth="1"/>
     <col min="14" max="14" width="22" customWidth="1"/>
     <col min="15" max="15" width="12" customWidth="1"/>
+    <col min="16" max="16" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -554,46 +552,52 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>46289</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K2" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="L2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="O2" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+      <c r="P2" s="2">
+        <v>46289</v>
       </c>
     </row>
   </sheetData>
@@ -602,9 +606,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
@@ -619,82 +623,89 @@
     <col min="11" max="11" width="19" customWidth="1"/>
     <col min="12" max="12" width="22" customWidth="1"/>
     <col min="13" max="13" width="13" customWidth="1"/>
+    <col min="14" max="14" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="2" t="s">
+      <c r="E1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>14</v>
       </c>
+      <c r="N1" s="3" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>46289</v>
       </c>
       <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" t="s">
         <v>34</v>
       </c>
-      <c r="C2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" t="s">
-        <v>29</v>
-      </c>
-      <c r="G2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H2" t="s">
-        <v>31</v>
-      </c>
-      <c r="I2" t="s">
-        <v>23</v>
-      </c>
-      <c r="J2" t="s">
-        <v>32</v>
-      </c>
       <c r="M2" t="s">
-        <v>33</v>
+        <v>35</v>
+      </c>
+      <c r="N2" s="2">
+        <v>46289</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: simplify import preview summary
</commit_message>
<xml_diff>
--- a/public/templates/OpsTracker_Import_Template.xlsx
+++ b/public/templates/OpsTracker_Import_Template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
   <si>
     <t>Date</t>
   </si>
@@ -35,6 +35,9 @@
     <t>Problem</t>
   </si>
   <si>
+    <t>Cause</t>
+  </si>
+  <si>
     <t>Category</t>
   </si>
   <si>
@@ -54,9 +57,6 @@
   </si>
   <si>
     <t>Assigned To</t>
-  </si>
-  <si>
-    <t>Accountable Person</t>
   </si>
   <si>
     <t>Remarks</t>
@@ -485,7 +485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -494,19 +494,19 @@
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="15" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="19" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="10" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="19" customWidth="1"/>
-    <col min="14" max="14" width="22" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="19" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="10" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="19" customWidth="1"/>
     <col min="15" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -556,7 +556,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>46289</v>
       </c>
@@ -575,22 +575,22 @@
       <c r="F2" t="s">
         <v>20</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>21</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>22</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>23</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>24</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>25</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>26</v>
       </c>
       <c r="O2" t="s">
@@ -612,18 +612,15 @@
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
-    <col min="6" max="6" width="29" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="19" customWidth="1"/>
-    <col min="12" max="12" width="22" customWidth="1"/>
-    <col min="13" max="13" width="13" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="29" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="19" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -634,39 +631,30 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="N1" s="3" t="s">
         <v>15</v>
       </c>
     </row>
@@ -678,33 +666,27 @@
         <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="E2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G2" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="H2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I2" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="J2" t="s">
-        <v>34</v>
-      </c>
-      <c r="M2" t="s">
         <v>35</v>
       </c>
-      <c r="N2" s="2">
+      <c r="K2" s="2">
         <v>46289</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: improve admin import ownership and accountability
</commit_message>
<xml_diff>
--- a/public/templates/OpsTracker_Import_Template.xlsx
+++ b/public/templates/OpsTracker_Import_Template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="37">
   <si>
     <t>Date</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t>Assigned To</t>
+  </si>
+  <si>
+    <t>Accountable Person</t>
   </si>
   <si>
     <t>Remarks</t>
@@ -502,8 +505,9 @@
     <col min="12" max="12" width="10" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="19" customWidth="1"/>
-    <col min="15" max="15" width="12" customWidth="1"/>
-    <col min="16" max="16" width="14" customWidth="1"/>
+    <col min="15" max="15" width="24" customWidth="1"/>
+    <col min="16" max="16" width="12" customWidth="1"/>
+    <col min="17" max="17" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
@@ -555,48 +559,51 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>46289</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O2" t="s">
         <v>27</v>
       </c>
-      <c r="P2" s="2">
+      <c r="P2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q2" s="2">
         <v>46289</v>
       </c>
     </row>
@@ -607,7 +614,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -619,11 +626,12 @@
     <col min="7" max="7" width="10" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="19" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="11" max="11" width="13" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -631,10 +639,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>9</v>
@@ -657,36 +665,39 @@
       <c r="K1" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="L1" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>46289</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H2" t="s">
-        <v>34</v>
-      </c>
-      <c r="J2" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L2" s="2">
         <v>46289</v>
       </c>
     </row>

</xml_diff>